<commit_message>
Merge invented 'San Joaquin Memorial HS' into existing portal SJM row
Portal already has a San Joaquin Memorial customer (c1773670554205).
This commit:
- INVENTED_PARENT_NAME_OVERRIDES renames my invented parent from
  "San Joaquin Memorial High School" to plain "San Joaquin Memorial"
  so the bulk insert can match on name.
- MERGE_INTO_EXISTING_PORTAL_PARENT: new dict exporting the mapping to
  a JSON file (data/customer-import/merge_into_existing_portal_parent.json)
  so the bulk-insert script can read it and use the existing portal id
  as parent_id for the cluster's subs, instead of creating a duplicate
  parent row.
- MANUAL_SUB_ASSIGNMENTS: pull 3 SJM orphans (Athletic Dept, Athletic
  Training, M Volleyball) under the cluster. Prefix demotion couldn't
  target them because "San Joaquin Memorial" doesn't end in a recognized
  institution suffix.

Net: SJM cluster now has 13 subs, all orphan SJM-named standalones gone.

https://claude.ai/code/session_01SY6MEd3PceMmndJjYjwk45
</commit_message>
<xml_diff>
--- a/data/customer-import/tier2_invented_parents.xlsx
+++ b/data/customer-import/tier2_invented_parents.xlsx
@@ -36291,12 +36291,12 @@
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>San Joaquin Memorial High School</t>
+          <t>San Joaquin Memorial</t>
         </is>
       </c>
       <c r="B405" s="2" t="inlineStr">
         <is>
-          <t>SJMHS</t>
+          <t>SJM</t>
         </is>
       </c>
       <c r="C405" s="2" t="inlineStr">
@@ -36386,7 +36386,7 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>San Joaquin Memorial High School</t>
+          <t>San Joaquin Memorial</t>
         </is>
       </c>
       <c r="E406" t="inlineStr"/>
@@ -36478,7 +36478,7 @@
       </c>
       <c r="D407" s="2" t="inlineStr">
         <is>
-          <t>San Joaquin Memorial High School</t>
+          <t>San Joaquin Memorial</t>
         </is>
       </c>
       <c r="E407" s="2" t="inlineStr"/>
@@ -36570,7 +36570,7 @@
       </c>
       <c r="D408" s="2" t="inlineStr">
         <is>
-          <t>San Joaquin Memorial High School</t>
+          <t>San Joaquin Memorial</t>
         </is>
       </c>
       <c r="E408" s="2" t="inlineStr"/>
@@ -36662,7 +36662,7 @@
       </c>
       <c r="D409" s="2" t="inlineStr">
         <is>
-          <t>San Joaquin Memorial High School</t>
+          <t>San Joaquin Memorial</t>
         </is>
       </c>
       <c r="E409" s="2" t="inlineStr"/>
@@ -36754,7 +36754,7 @@
       </c>
       <c r="D410" s="2" t="inlineStr">
         <is>
-          <t>San Joaquin Memorial High School</t>
+          <t>San Joaquin Memorial</t>
         </is>
       </c>
       <c r="E410" s="2" t="inlineStr"/>
@@ -36846,7 +36846,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>San Joaquin Memorial High School</t>
+          <t>San Joaquin Memorial</t>
         </is>
       </c>
       <c r="E411" t="inlineStr"/>
@@ -36938,7 +36938,7 @@
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>San Joaquin Memorial High School</t>
+          <t>San Joaquin Memorial</t>
         </is>
       </c>
       <c r="E412" t="inlineStr"/>
@@ -37030,7 +37030,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>San Joaquin Memorial High School</t>
+          <t>San Joaquin Memorial</t>
         </is>
       </c>
       <c r="E413" t="inlineStr"/>
@@ -37122,7 +37122,7 @@
       </c>
       <c r="D414" s="2" t="inlineStr">
         <is>
-          <t>San Joaquin Memorial High School</t>
+          <t>San Joaquin Memorial</t>
         </is>
       </c>
       <c r="E414" s="2" t="inlineStr"/>
@@ -37214,7 +37214,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>San Joaquin Memorial High School</t>
+          <t>San Joaquin Memorial</t>
         </is>
       </c>
       <c r="E415" t="inlineStr"/>
@@ -37306,7 +37306,7 @@
       </c>
       <c r="D416" s="2" t="inlineStr">
         <is>
-          <t>San Joaquin Memorial High School</t>
+          <t>San Joaquin Memorial</t>
         </is>
       </c>
       <c r="E416" s="2" t="inlineStr"/>
@@ -37398,7 +37398,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>San Joaquin Memorial High School</t>
+          <t>San Joaquin Memorial</t>
         </is>
       </c>
       <c r="E417" t="inlineStr"/>
@@ -37490,7 +37490,7 @@
       </c>
       <c r="D418" s="2" t="inlineStr">
         <is>
-          <t>San Joaquin Memorial High School</t>
+          <t>San Joaquin Memorial</t>
         </is>
       </c>
       <c r="E418" s="2" t="inlineStr"/>
@@ -50345,7 +50345,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>San Joaquin Memorial High School</t>
+          <t>San Joaquin Memorial</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">

</xml_diff>